<commit_message>
Update ETF data and clean old Excel files
</commit_message>
<xml_diff>
--- a/etf_holdings/2026-08-25_00403A_full_holdings.xlsx
+++ b/etf_holdings/2026-08-25_00403A_full_holdings.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -509,25 +509,25 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>-1.45%2375</t>
+          <t>+1.05%2400</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>-1.45%</t>
+          <t>+1.05%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2375</v>
+        <v>2400</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>17.19%12,000,000</t>
+          <t>17.14%12,000,000</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>17.19%</t>
+          <t>17.14%</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>-0.25%</t>
+          <t>+0.18%</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -570,25 +570,25 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>-4.4%5430</t>
+          <t>+3.04%5595</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>-4.4%</t>
+          <t>+3.04%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>5430</v>
+        <v>5595</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>5.53%1,690,000</t>
+          <t>5.63%1,690,000</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>5.63%</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -596,7 +596,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>-0.25%</t>
+          <t>+0.17%</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -631,25 +631,25 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.92%1075</t>
+          <t>+1.86%1095</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-0.92%</t>
+          <t>+1.86%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1075</v>
+        <v>1095</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5.49%8,460,000</t>
+          <t>5.51%8,460,000</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>5.51%</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -657,7 +657,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>+0.10%</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -692,33 +692,33 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.35%2855</t>
+          <t>+3.33%2950</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>-0.35%</t>
+          <t>+3.33%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2855</v>
+        <v>2950</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5.17%3,000,000</t>
+          <t>5.44%3,100,000</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5.17%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>3000000</v>
+        <v>3100000</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>+0.18%</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -753,25 +753,25 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.66%3765</t>
+          <t>-0.8%3735</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>-0.8%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>3765</v>
+        <v>3735</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>4.79%2,110,000</t>
+          <t>4.69%2,110,000</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>4.69%</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -779,7 +779,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -814,25 +814,25 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>+6.01%123.5</t>
+          <t>+1.21%125</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>+6.01%</t>
+          <t>+1.21%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>123.5</v>
+        <v>125</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4.47%60,000,000</t>
+          <t>4.46%60,000,000</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>4.47%</t>
+          <t>4.46%</t>
         </is>
       </c>
       <c r="K7" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>+0.25%</t>
+          <t>+0.05%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -875,25 +875,25 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>+1.83%5565</t>
+          <t>+0.63%5600</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>+1.83%</t>
+          <t>+0.63%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>5565</v>
+        <v>5600</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3.69%1,100,000</t>
+          <t>3.67%1,100,000</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3.69%</t>
+          <t>3.67%</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -901,7 +901,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>+0.07%</t>
+          <t>+0.02%</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -936,25 +936,25 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>-4.45%5155</t>
+          <t>+0.97%5205</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-4.45%</t>
+          <t>+0.97%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>5155</v>
+        <v>5205</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3.36%1,080,000</t>
+          <t>3.34%1,080,000</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>3.36%</t>
+          <t>3.34%</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>+0.03%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -997,25 +997,25 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-0.54%551</t>
+          <t>-1.27%544</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-0.54%</t>
+          <t>-1.27%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>551</v>
+        <v>544</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3.25%9,785,000</t>
+          <t>3.17%9,785,000</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1058,25 +1058,25 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.86%1735</t>
+          <t>-1.44%1710</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-0.86%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1735</v>
+        <v>1710</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3.18%3,040,000</t>
+          <t>3.09%3,040,000</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3.18%</t>
+          <t>3.09%</t>
         </is>
       </c>
       <c r="K11" t="n">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1114,38 +1114,38 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2345智邦</t>
+          <t>3711日月光投控</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>+1.72%2070</t>
+          <t>-0.17%591</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>+1.72%</t>
+          <t>-0.17%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>2070</v>
+        <v>591</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2.88%2,307,000</t>
+          <t>2.81%8,000,000</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2.88%</t>
+          <t>2.81%</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>2307000</v>
+        <v>8000000</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>+0.05%</t>
+          <t>-0.00%</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1175,38 +1175,38 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3711日月光投控</t>
+          <t>2345智邦</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>+0.85%592</t>
+          <t>-1.93%2030</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>+0.85%</t>
+          <t>-1.93%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>592</v>
+        <v>2030</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2.86%8,000,000</t>
+          <t>2.79%2,307,000</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2.86%</t>
+          <t>2.79%</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>8000000</v>
+        <v>2307000</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>+0.02%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1241,33 +1241,33 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>+0.72%6300</t>
+          <t>+2.22%6440</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>+0.72%</t>
+          <t>+2.22%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>6300</v>
+        <v>6440</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.32%610,000</t>
+          <t>2.41%630,000</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2.32%</t>
+          <t>2.41%</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>610000</v>
+        <v>630000</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>+0.02%</t>
+          <t>+0.05%</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1297,38 +1297,38 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3189景碩</t>
+          <t>3008大立光</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-2.1%794</t>
+          <t>+6.22%5720</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-2.1%</t>
+          <t>+6.22%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>794</v>
+        <v>5720</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2.04%4,250,000</t>
+          <t>2.13%626,000</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2.04%</t>
+          <t>2.13%</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>4250000</v>
+        <v>626000</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>+0.13%</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:55</t>
+          <t>2026-08-25 17:37:30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1358,38 +1358,38 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3008大立光</t>
+          <t>3189景碩</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>-4.01%5385</t>
+          <t>+5.16%835</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>-4.01%</t>
+          <t>+5.16%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>5385</v>
+        <v>835</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.03%626,000</t>
+          <t>2.11%4,250,000</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2.03%</t>
+          <t>2.11%</t>
         </is>
       </c>
       <c r="K16" t="n">
-        <v>626000</v>
+        <v>4250000</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>-0.08%</t>
+          <t>+0.10%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1424,25 +1424,25 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>-4.2%5365</t>
+          <t>+3.82%5570</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-4.2%</t>
+          <t>+3.82%</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>5365</v>
+        <v>5570</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1.97%610,000</t>
+          <t>2.02%610,000</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>1.97%</t>
+          <t>2.02%</t>
         </is>
       </c>
       <c r="K17" t="n">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>+0.07%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1485,25 +1485,25 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0%1135</t>
+          <t>+2.2%1160</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>+2.2%</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1135</v>
+        <v>1160</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1.81%2,640,000</t>
+          <t>1.82%2,640,000</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>1.81%</t>
+          <t>1.82%</t>
         </is>
       </c>
       <c r="K18" t="n">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>+0.04%</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1541,38 +1541,38 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6488環球晶</t>
+          <t>5274信驊</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>+7.33%1010</t>
+          <t>+1.89%15400</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>+7.33%</t>
+          <t>+1.89%</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1010</v>
+        <v>15400</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.71%2,800,000</t>
+          <t>1.64%179,500</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>1.71%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>2800000</v>
+        <v>179500</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>+0.12%</t>
+          <t>+0.03%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1602,38 +1602,38 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>5274信驊</t>
+          <t>6488環球晶</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>-1.53%15115</t>
+          <t>-2.97%980</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>-1.53%</t>
+          <t>-2.97%</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>15115</v>
+        <v>980</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1.64%179,500</t>
+          <t>1.63%2,800,000</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.63%</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>179500</v>
+        <v>2800000</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1668,16 +1668,16 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-2.21%177</t>
+          <t>+1.13%179</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-2.21%</t>
+          <t>+1.13%</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>+0.02%</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1729,25 +1729,25 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>-2.68%1455</t>
+          <t>+2.06%1485</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-2.68%</t>
+          <t>+2.06%</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1455</v>
+        <v>1485</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.58%1,800,000</t>
+          <t>1.59%1,800,000</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>1.58%</t>
+          <t>1.59%</t>
         </is>
       </c>
       <c r="K22" t="n">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>+0.03%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1790,16 +1790,16 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>-9.89%2050</t>
+          <t>+1.22%2075</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-9.89%</t>
+          <t>+1.22%</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>2050</v>
+        <v>2075</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>+0.02%</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1846,38 +1846,38 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2360致茂</t>
+          <t>8996高力</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>-1.43%2070</t>
+          <t>+6.11%1215</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>-1.43%</t>
+          <t>+6.11%</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>2070</v>
+        <v>1215</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1.25%1,000,000</t>
+          <t>1.24%1,720,000</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>1.25%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="K24" t="n">
-        <v>1000000</v>
+        <v>1720000</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>+0.07%</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1907,38 +1907,38 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>8996高力</t>
+          <t>2360致茂</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>+5.05%1145</t>
+          <t>-5.07%1965</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>+5.05%</t>
+          <t>-5.07%</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>1145</v>
+        <v>1965</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1.10%1,600,000</t>
+          <t>1.17%1,000,000</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>1.17%</t>
         </is>
       </c>
       <c r="K25" t="n">
-        <v>1600000</v>
+        <v>1000000</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>+0.05%</t>
+          <t>-0.06%</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1973,33 +1973,33 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>-6.25%180</t>
+          <t>+4.72%188.5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>-6.25%</t>
+          <t>+4.72%</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>180</v>
+        <v>188.5</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>0.98%9,000,000</t>
+          <t>1.12%10,000,000</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>0.98%</t>
+          <t>1.12%</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>9000000</v>
+        <v>10000000</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>+0.05%</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2034,16 +2034,16 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>+0.75%269.5</t>
+          <t>+1.48%273.5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>+0.75%</t>
+          <t>+1.48%</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>269.5</v>
+        <v>273.5</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2095,33 +2095,33 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>-3.12%1710</t>
+          <t>+7.89%1845</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>-3.12%</t>
+          <t>+7.89%</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1710</v>
+        <v>1845</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>0.72%700,000</t>
+          <t>0.86%780,000</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>0.72%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="K28" t="n">
-        <v>700000</v>
+        <v>780000</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>+0.06%</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2151,38 +2151,38 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3450聯鈞</t>
+          <t>7769鴻勁</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>-7.99%507</t>
+          <t>-0.72%6210</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>-7.99%</t>
+          <t>-0.72%</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>507</v>
+        <v>6210</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>0.55%1,800,000</t>
+          <t>0.48%130,000</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>0.55%</t>
+          <t>0.48%</t>
         </is>
       </c>
       <c r="K29" t="n">
-        <v>1800000</v>
+        <v>130000</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>-0.00%</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2212,38 +2212,38 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>3533嘉澤</t>
+          <t>2317鴻海</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>+0.94%1610</t>
+          <t>-0.21%243</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>+0.94%</t>
+          <t>-0.21%</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1610</v>
+        <v>243</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>0.51%525,000</t>
+          <t>0.46%3,200,000</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="K30" t="n">
-        <v>525000</v>
+        <v>3200000</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.00%</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:56</t>
+          <t>2026-08-25 17:37:31</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2273,38 +2273,38 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>7769鴻勁</t>
+          <t>3211順達</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>-2.34%6255</t>
+          <t>+1.53%331</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>-2.34%</t>
+          <t>+1.53%</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>6255</v>
+        <v>331</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>0.49%130,000</t>
+          <t>0.39%2,000,000</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>0.49%</t>
+          <t>0.39%</t>
         </is>
       </c>
       <c r="K31" t="n">
-        <v>130000</v>
+        <v>2000000</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>+0.01%</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2334,38 +2334,38 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2317鴻海</t>
+          <t>2337旺宏</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>-0.81%243.5</t>
+          <t>-1.61%122</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>-0.81%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>243.5</v>
+        <v>122</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>0.47%3,200,000</t>
+          <t>0.33%4,500,000</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="K32" t="n">
-        <v>3200000</v>
+        <v>4500000</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>-0.00%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2395,38 +2395,38 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>3211順達</t>
+          <t>3583辛耘</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>-6.99%326</t>
+          <t>+0.73%693</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>-6.99%</t>
+          <t>+0.73%</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>326</v>
+        <v>693</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>0.39%2,000,000</t>
+          <t>0.33%800,000</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>0.39%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2000000</v>
+        <v>800000</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>-0.03%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2456,38 +2456,38 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2337旺宏</t>
+          <t>2059川湖</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>+1.22%124</t>
+          <t>-0.87%14285</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>+1.22%</t>
+          <t>-0.87%</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>124</v>
+        <v>14285</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>0.34%4,500,000</t>
+          <t>0.30%35,000</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.30%</t>
         </is>
       </c>
       <c r="K34" t="n">
-        <v>4500000</v>
+        <v>35000</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.00%</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2517,38 +2517,38 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>3583辛耘</t>
+          <t>3533嘉澤</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>-2.27%688</t>
+          <t>-0.31%1605</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>-2.27%</t>
+          <t>-0.31%</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>688</v>
+        <v>1605</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>0.33%800,000</t>
+          <t>0.29%300,000</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.29%</t>
         </is>
       </c>
       <c r="K35" t="n">
-        <v>800000</v>
+        <v>300000</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.00%</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2578,34 +2578,34 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2059川湖</t>
+          <t>6442光聖</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>+7.66%14410</t>
+          <t>+9.93%1605</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>+7.66%</t>
+          <t>+9.93%</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>14410</v>
+        <v>1605</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>0.30%35,000</t>
+          <t>0.21%225,000</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>0.21%</t>
         </is>
       </c>
       <c r="K36" t="n">
-        <v>35000</v>
+        <v>225000</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2639,25 +2639,25 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>6442光聖</t>
+          <t>8358金居</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>-4.26%1460</t>
+          <t>+2.88%429</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>-4.26%</t>
+          <t>+2.88%</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1460</v>
+        <v>429</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>0.20%225,000</t>
+          <t>0.20%800,000</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2666,11 +2666,11 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>225000</v>
+        <v>800000</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>+0.01%</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2700,38 +2700,38 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>8358金居</t>
+          <t>1560中砂</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>-4.36%417</t>
+          <t>-0.44%677</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>-4.36%</t>
+          <t>-0.44%</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>417</v>
+        <v>677</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>0.20%800,000</t>
+          <t>0.16%393,000</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="K38" t="n">
-        <v>800000</v>
+        <v>393000</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.00%</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2761,38 +2761,38 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>4966譜瑞-KY</t>
+          <t>2404漢唐</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>-1.59%557</t>
+          <t>+0.47%1070</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>-1.59%</t>
+          <t>+0.47%</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>557</v>
+        <v>1070</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>0.17%500,000</t>
+          <t>0.16%250,000</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="K39" t="n">
-        <v>500000</v>
+        <v>250000</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>-0.00%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2822,34 +2822,34 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1560中砂</t>
+          <t>4958臻鼎-KY</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>+0.15%680</t>
+          <t>+1.95%444</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>+0.15%</t>
+          <t>+1.95%</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>680</v>
+        <v>444</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>0.16%393,000</t>
+          <t>0.13%500,000</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="K40" t="n">
-        <v>393000</v>
+        <v>500000</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2883,38 +2883,38 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2404漢唐</t>
+          <t>3450聯鈞</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>+0.47%1065</t>
+          <t>+5.13%533</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>+0.47%</t>
+          <t>+5.13%</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1065</v>
+        <v>533</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>0.16%250,000</t>
+          <t>0.13%400,000</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="K41" t="n">
-        <v>250000</v>
+        <v>400000</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>+0.01%</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2944,38 +2944,38 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4958臻鼎-KY</t>
+          <t>1717長興</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>-1.25%435.5</t>
+          <t>+0.56%71.7</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>-1.25%</t>
+          <t>+0.56%</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>435.5</v>
+        <v>71.7</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>0.13%500,000</t>
+          <t>0.11%2,500,000</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="K42" t="n">
-        <v>500000</v>
+        <v>2500000</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>-0.00%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3005,38 +3005,38 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1717長興</t>
+          <t>3264欣銓</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>-0.42%71.3</t>
+          <t>+3.65%213</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>-0.42%</t>
+          <t>+3.65%</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>71.3</v>
+        <v>213</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>0.11%2,500,000</t>
+          <t>0.09%700,000</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>0.09%</t>
         </is>
       </c>
       <c r="K43" t="n">
-        <v>2500000</v>
+        <v>700000</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>-0.00%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3066,38 +3066,38 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>3264欣銓</t>
+          <t>4966譜瑞-KY</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>+1.23%205.5</t>
+          <t>-0.18%556</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>+1.23%</t>
+          <t>-0.18%</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>205.5</v>
+        <v>556</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>0.09%700,000</t>
+          <t>0.07%220,000</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>0.09%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="K44" t="n">
-        <v>700000</v>
+        <v>220000</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.00%</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3132,16 +3132,16 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>-2.12%230.5</t>
+          <t>+1.3%233.5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>+1.3%</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>230.5</v>
+        <v>233.5</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>-0.00%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:57</t>
+          <t>2026-08-25 17:37:32</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3193,16 +3193,16 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>-6.03%381.5</t>
+          <t>+9.96%419.5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>-6.03%</t>
+          <t>+9.96%</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>381.5</v>
+        <v>419.5</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>-0.00%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:59</t>
+          <t>2026-08-25 17:37:34</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3254,16 +3254,16 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>+2.89%2135</t>
+          <t>-2.34%2085</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>+2.89%</t>
+          <t>-2.34%</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>2135</v>
+        <v>2085</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:59</t>
+          <t>2026-08-25 17:37:34</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3315,16 +3315,16 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>+0.51%493</t>
+          <t>-3.25%477</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>+0.51%</t>
+          <t>-3.25%</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>493</v>
+        <v>477</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:59</t>
+          <t>2026-08-25 17:37:34</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3376,16 +3376,16 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>-1.58%343.5</t>
+          <t>+0.58%345.5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>-1.58%</t>
+          <t>+0.58%</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>343.5</v>
+        <v>345.5</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:59</t>
+          <t>2026-08-25 17:37:34</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>-0.33%151</t>
+          <t>-0.33%150.5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3446,7 +3446,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>151</v>
+        <v>150.5</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-08-25 10:24:59</t>
+          <t>2026-08-25 17:37:34</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3498,16 +3498,16 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>+0.75%134</t>
+          <t>+2.24%137</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>+0.75%</t>
+          <t>+2.24%</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>

</xml_diff>